<commit_message>
continuing script to handle multiple table format
</commit_message>
<xml_diff>
--- a/data/tracker_files/file_status_record_2026-02-27.xlsx
+++ b/data/tracker_files/file_status_record_2026-02-27.xlsx
@@ -14,6 +14,7 @@
   <sheets>
     <sheet name="Sheet" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
+    <sheet name="Completed Pipelines" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet!$A$1:$J$131</definedName>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1715" uniqueCount="392">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1852" uniqueCount="403">
   <si>
     <t>Pipeline</t>
   </si>
@@ -1190,16 +1191,49 @@
     <t>Inc</t>
   </si>
   <si>
-    <t>No Pipeline</t>
-  </si>
-  <si>
-    <t>No Pipeline and Date</t>
-  </si>
-  <si>
-    <t>No Date</t>
-  </si>
-  <si>
-    <t>NoDate</t>
+    <t>Extracted data</t>
+  </si>
+  <si>
+    <t>desination name</t>
+  </si>
+  <si>
+    <t>Pony Express Page 8</t>
+  </si>
+  <si>
+    <t>Yes (partial)</t>
+  </si>
+  <si>
+    <t>FROM: TO: RATE:</t>
+  </si>
+  <si>
+    <t>Origin Point</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Destination Point</t>
+  </si>
+  <si>
+    <t>Committed Shipper Rate</t>
+  </si>
+  <si>
+    <t>Uncommitted</t>
+  </si>
+  <si>
+    <t>UNCOMMITTED</t>
+  </si>
+  <si>
+    <t>COMMITTED</t>
+  </si>
+  <si>
+    <t>FROM</t>
+  </si>
+  <si>
+    <t>TO</t>
+  </si>
+  <si>
+    <t>Maximum Rate</t>
+  </si>
+  <si>
+    <t>Volume Discount Rate</t>
   </si>
 </sst>
 </file>
@@ -5035,17 +5069,19 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr filterMode="1"/>
-  <dimension ref="A1:X75"/>
+  <dimension ref="A1:AD75"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="34.28515625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="19" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="14.42578125" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="18" max="21" width="9.140625" customWidth="1"/>
+    <col min="28" max="28" width="22.7109375" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="24.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -5088,8 +5124,14 @@
       <c r="R1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:24" hidden="1" x14ac:dyDescent="0.25">
+      <c r="V1" t="s">
+        <v>388</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>201</v>
       </c>
@@ -5132,8 +5174,11 @@
       <c r="P2">
         <v>2</v>
       </c>
-    </row>
-    <row r="3" spans="1:24" hidden="1" x14ac:dyDescent="0.25">
+      <c r="V2" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="3" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>173</v>
       </c>
@@ -5177,7 +5222,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:24" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>274</v>
       </c>
@@ -5221,7 +5266,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:24" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>297</v>
       </c>
@@ -5265,7 +5310,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>47</v>
       </c>
@@ -5320,8 +5365,20 @@
       <c r="U6" t="s">
         <v>362</v>
       </c>
-    </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="V6" t="s">
+        <v>331</v>
+      </c>
+      <c r="AB6" t="s">
+        <v>360</v>
+      </c>
+      <c r="AC6" t="s">
+        <v>361</v>
+      </c>
+      <c r="AD6" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="7" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>79</v>
       </c>
@@ -5376,8 +5433,20 @@
       <c r="U7" t="s">
         <v>362</v>
       </c>
-    </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="V7" t="s">
+        <v>329</v>
+      </c>
+      <c r="AB7" t="s">
+        <v>365</v>
+      </c>
+      <c r="AC7" t="s">
+        <v>363</v>
+      </c>
+      <c r="AD7" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="8" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>13</v>
       </c>
@@ -5432,8 +5501,20 @@
       <c r="U8" t="s">
         <v>362</v>
       </c>
-    </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="V8" t="s">
+        <v>391</v>
+      </c>
+      <c r="AB8" t="s">
+        <v>360</v>
+      </c>
+      <c r="AC8" t="s">
+        <v>361</v>
+      </c>
+      <c r="AD8" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="9" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>97</v>
       </c>
@@ -5488,11 +5569,23 @@
       <c r="U9" t="s">
         <v>364</v>
       </c>
-      <c r="X9" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="V9" t="s">
+        <v>331</v>
+      </c>
+      <c r="W9" t="s">
+        <v>389</v>
+      </c>
+      <c r="AB9" t="s">
+        <v>366</v>
+      </c>
+      <c r="AC9" t="s">
+        <v>367</v>
+      </c>
+      <c r="AD9" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="10" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>115</v>
       </c>
@@ -5547,8 +5640,20 @@
       <c r="U10" t="s">
         <v>368</v>
       </c>
-    </row>
-    <row r="11" spans="1:24" hidden="1" x14ac:dyDescent="0.25">
+      <c r="V10" t="s">
+        <v>331</v>
+      </c>
+      <c r="AB10" t="s">
+        <v>372</v>
+      </c>
+      <c r="AC10" t="s">
+        <v>373</v>
+      </c>
+      <c r="AD10" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="11" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>101</v>
       </c>
@@ -5591,8 +5696,11 @@
       <c r="P11" t="s">
         <v>350</v>
       </c>
-    </row>
-    <row r="12" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="V11" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="12" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>89</v>
       </c>
@@ -5635,8 +5743,11 @@
       <c r="P12">
         <v>2</v>
       </c>
-    </row>
-    <row r="13" spans="1:24" hidden="1" x14ac:dyDescent="0.25">
+      <c r="V12" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="13" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>45</v>
       </c>
@@ -5668,7 +5779,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="14" spans="1:24" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>94</v>
       </c>
@@ -5712,7 +5823,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:24" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>133</v>
       </c>
@@ -5753,7 +5864,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="16" spans="1:24" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>162</v>
       </c>
@@ -5796,8 +5907,14 @@
       <c r="P16">
         <v>2</v>
       </c>
-    </row>
-    <row r="17" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="V16" t="s">
+        <v>329</v>
+      </c>
+      <c r="Y16" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="17" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>266</v>
       </c>
@@ -5852,8 +5969,20 @@
       <c r="U17" t="s">
         <v>362</v>
       </c>
-    </row>
-    <row r="18" spans="1:24" hidden="1" x14ac:dyDescent="0.25">
+      <c r="V17" t="s">
+        <v>331</v>
+      </c>
+      <c r="AB17" t="s">
+        <v>384</v>
+      </c>
+      <c r="AC17" t="s">
+        <v>385</v>
+      </c>
+      <c r="AD17" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="18" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>254</v>
       </c>
@@ -5881,11 +6010,32 @@
       <c r="J18" t="s">
         <v>335</v>
       </c>
-      <c r="K18" t="s">
-        <v>351</v>
-      </c>
-    </row>
-    <row r="19" spans="1:24" hidden="1" x14ac:dyDescent="0.25">
+      <c r="L18" t="s">
+        <v>346</v>
+      </c>
+      <c r="M18" t="s">
+        <v>343</v>
+      </c>
+      <c r="N18" t="s">
+        <v>344</v>
+      </c>
+      <c r="R18" t="s">
+        <v>370</v>
+      </c>
+      <c r="S18" t="s">
+        <v>360</v>
+      </c>
+      <c r="T18" t="s">
+        <v>361</v>
+      </c>
+      <c r="U18" t="s">
+        <v>362</v>
+      </c>
+      <c r="V18" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="19" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>84</v>
       </c>
@@ -5929,7 +6079,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:24" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>325</v>
       </c>
@@ -5973,7 +6123,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:24" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>226</v>
       </c>
@@ -6017,7 +6167,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="1:24" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>302</v>
       </c>
@@ -6060,8 +6210,23 @@
       <c r="P22" t="s">
         <v>355</v>
       </c>
-    </row>
-    <row r="23" spans="1:24" hidden="1" x14ac:dyDescent="0.25">
+      <c r="V22" t="s">
+        <v>331</v>
+      </c>
+      <c r="Y22" t="s">
+        <v>393</v>
+      </c>
+      <c r="Z22" t="s">
+        <v>394</v>
+      </c>
+      <c r="AA22" t="s">
+        <v>396</v>
+      </c>
+      <c r="AB22" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="23" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>312</v>
       </c>
@@ -6104,8 +6269,23 @@
       <c r="P23">
         <v>25</v>
       </c>
-    </row>
-    <row r="24" spans="1:24" hidden="1" x14ac:dyDescent="0.25">
+      <c r="V23" t="s">
+        <v>331</v>
+      </c>
+      <c r="Y23" t="s">
+        <v>393</v>
+      </c>
+      <c r="Z23" t="s">
+        <v>394</v>
+      </c>
+      <c r="AA23" t="s">
+        <v>396</v>
+      </c>
+      <c r="AB23" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="24" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>232</v>
       </c>
@@ -6148,8 +6328,23 @@
       <c r="P24">
         <v>3</v>
       </c>
-    </row>
-    <row r="25" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="V24" t="s">
+        <v>331</v>
+      </c>
+      <c r="Y24" t="s">
+        <v>360</v>
+      </c>
+      <c r="Z24" t="s">
+        <v>361</v>
+      </c>
+      <c r="AA24" t="s">
+        <v>396</v>
+      </c>
+      <c r="AB24" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="25" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>148</v>
       </c>
@@ -6204,11 +6399,20 @@
       <c r="U25" t="s">
         <v>362</v>
       </c>
-      <c r="X25" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="26" spans="1:24" hidden="1" x14ac:dyDescent="0.25">
+      <c r="V25" t="s">
+        <v>331</v>
+      </c>
+      <c r="AB25" t="s">
+        <v>375</v>
+      </c>
+      <c r="AC25" t="s">
+        <v>376</v>
+      </c>
+      <c r="AD25" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="26" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>55</v>
       </c>
@@ -6252,7 +6456,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="27" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>119</v>
       </c>
@@ -6295,8 +6499,26 @@
       <c r="P27">
         <v>8</v>
       </c>
-    </row>
-    <row r="28" spans="1:24" hidden="1" x14ac:dyDescent="0.25">
+      <c r="V27" t="s">
+        <v>331</v>
+      </c>
+      <c r="Y27" t="s">
+        <v>384</v>
+      </c>
+      <c r="Z27" t="s">
+        <v>367</v>
+      </c>
+      <c r="AA27" t="s">
+        <v>397</v>
+      </c>
+      <c r="AB27" t="s">
+        <v>398</v>
+      </c>
+      <c r="AC27" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="28" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>234</v>
       </c>
@@ -6339,8 +6561,23 @@
       <c r="P28">
         <v>11</v>
       </c>
-    </row>
-    <row r="29" spans="1:24" hidden="1" x14ac:dyDescent="0.25">
+      <c r="V28" t="s">
+        <v>331</v>
+      </c>
+      <c r="Y28" t="s">
+        <v>399</v>
+      </c>
+      <c r="Z28" t="s">
+        <v>400</v>
+      </c>
+      <c r="AA28" t="s">
+        <v>401</v>
+      </c>
+      <c r="AB28" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="29" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>237</v>
       </c>
@@ -6372,7 +6609,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="30" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>239</v>
       </c>
@@ -6427,8 +6664,11 @@
       <c r="U30" t="s">
         <v>374</v>
       </c>
-    </row>
-    <row r="31" spans="1:24" hidden="1" x14ac:dyDescent="0.25">
+      <c r="V30" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="31" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>58</v>
       </c>
@@ -6472,7 +6712,7 @@
         <v>46297</v>
       </c>
     </row>
-    <row r="32" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>243</v>
       </c>
@@ -6527,8 +6767,11 @@
       <c r="U32" t="s">
         <v>362</v>
       </c>
-    </row>
-    <row r="33" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="V32" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="33" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>245</v>
       </c>
@@ -6583,8 +6826,11 @@
       <c r="U33" t="s">
         <v>362</v>
       </c>
-    </row>
-    <row r="34" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="V33" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="34" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>138</v>
       </c>
@@ -6639,8 +6885,11 @@
       <c r="U34" t="s">
         <v>374</v>
       </c>
-    </row>
-    <row r="35" spans="1:24" hidden="1" x14ac:dyDescent="0.25">
+      <c r="V34" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="35" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>241</v>
       </c>
@@ -6672,7 +6921,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="36" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>110</v>
       </c>
@@ -6727,8 +6976,11 @@
       <c r="U36" t="s">
         <v>362</v>
       </c>
-    </row>
-    <row r="37" spans="1:24" hidden="1" x14ac:dyDescent="0.25">
+      <c r="V36" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="37" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>251</v>
       </c>
@@ -6760,7 +7012,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="38" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>92</v>
       </c>
@@ -6815,8 +7067,11 @@
       <c r="U38" t="s">
         <v>379</v>
       </c>
-    </row>
-    <row r="39" spans="1:24" hidden="1" x14ac:dyDescent="0.25">
+      <c r="V38" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="39" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>144</v>
       </c>
@@ -6860,7 +7115,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="40" spans="1:24" hidden="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>146</v>
       </c>
@@ -6892,7 +7147,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="41" spans="1:24" hidden="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>131</v>
       </c>
@@ -6924,7 +7179,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="42" spans="1:24" hidden="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>136</v>
       </c>
@@ -6956,7 +7211,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="43" spans="1:24" hidden="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>322</v>
       </c>
@@ -6988,7 +7243,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="44" spans="1:24" hidden="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>74</v>
       </c>
@@ -7020,7 +7275,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="45" spans="1:24" hidden="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>178</v>
       </c>
@@ -7064,7 +7319,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="46" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>129</v>
       </c>
@@ -7093,7 +7348,7 @@
         <v>333</v>
       </c>
       <c r="L46" t="s">
-        <v>346</v>
+        <v>390</v>
       </c>
       <c r="M46" t="s">
         <v>343</v>
@@ -7119,8 +7374,11 @@
       <c r="U46" t="s">
         <v>368</v>
       </c>
-    </row>
-    <row r="47" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="V46" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="47" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>288</v>
       </c>
@@ -7175,11 +7433,11 @@
       <c r="U47" t="s">
         <v>379</v>
       </c>
-      <c r="X47" t="s">
-        <v>391</v>
-      </c>
-    </row>
-    <row r="48" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="V47" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="48" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>214</v>
       </c>
@@ -7234,11 +7492,11 @@
       <c r="U48" t="s">
         <v>368</v>
       </c>
-      <c r="X48" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="49" spans="1:24" hidden="1" x14ac:dyDescent="0.25">
+      <c r="V48" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="49" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>219</v>
       </c>
@@ -7270,7 +7528,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="50" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>206</v>
       </c>
@@ -7325,8 +7583,11 @@
       <c r="U50" t="s">
         <v>368</v>
       </c>
-    </row>
-    <row r="51" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="V50" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="51" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>216</v>
       </c>
@@ -7381,11 +7642,11 @@
       <c r="U51" t="s">
         <v>368</v>
       </c>
-      <c r="X51" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="52" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="V51" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="52" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>211</v>
       </c>
@@ -7440,11 +7701,11 @@
       <c r="U52" t="s">
         <v>368</v>
       </c>
-      <c r="X52" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="53" spans="1:24" hidden="1" x14ac:dyDescent="0.25">
+      <c r="V52" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="53" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>208</v>
       </c>
@@ -7476,7 +7737,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="54" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>283</v>
       </c>
@@ -7529,7 +7790,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="55" spans="1:24" hidden="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>33</v>
       </c>
@@ -7573,7 +7834,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="56" spans="1:24" hidden="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>123</v>
       </c>
@@ -7617,7 +7878,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="57" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>181</v>
       </c>
@@ -7672,8 +7933,11 @@
       <c r="U57" t="s">
         <v>362</v>
       </c>
-    </row>
-    <row r="58" spans="1:24" hidden="1" x14ac:dyDescent="0.25">
+      <c r="V57" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="58" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>318</v>
       </c>
@@ -7717,7 +7981,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="59" spans="1:24" hidden="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>170</v>
       </c>
@@ -7761,7 +8025,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="60" spans="1:24" hidden="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>323</v>
       </c>
@@ -7805,7 +8069,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="61" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>199</v>
       </c>
@@ -7860,8 +8124,11 @@
       <c r="U61" t="s">
         <v>362</v>
       </c>
-    </row>
-    <row r="62" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="V61" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="62" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>307</v>
       </c>
@@ -7913,11 +8180,11 @@
       <c r="U62" t="s">
         <v>379</v>
       </c>
-      <c r="X62" t="s">
-        <v>389</v>
-      </c>
-    </row>
-    <row r="63" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="V62" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="63" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>277</v>
       </c>
@@ -7972,8 +8239,11 @@
       <c r="U63" t="s">
         <v>374</v>
       </c>
-    </row>
-    <row r="64" spans="1:24" hidden="1" x14ac:dyDescent="0.25">
+      <c r="V63" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="64" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>176</v>
       </c>
@@ -8005,7 +8275,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="65" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>99</v>
       </c>
@@ -8060,8 +8330,11 @@
       <c r="U65" t="s">
         <v>374</v>
       </c>
-    </row>
-    <row r="66" spans="1:24" hidden="1" x14ac:dyDescent="0.25">
+      <c r="V65" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="66" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>121</v>
       </c>
@@ -8105,7 +8378,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="67" spans="1:24" hidden="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>142</v>
       </c>
@@ -8149,7 +8422,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="68" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>159</v>
       </c>
@@ -8204,11 +8477,11 @@
       <c r="U68" t="s">
         <v>379</v>
       </c>
-      <c r="X68" t="s">
-        <v>390</v>
-      </c>
-    </row>
-    <row r="69" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="V68" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="69" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>87</v>
       </c>
@@ -8263,8 +8536,11 @@
       <c r="U69" t="s">
         <v>379</v>
       </c>
-    </row>
-    <row r="70" spans="1:24" hidden="1" x14ac:dyDescent="0.25">
+      <c r="V69" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="70" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>328</v>
       </c>
@@ -8296,7 +8572,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="71" spans="1:24" hidden="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>256</v>
       </c>
@@ -8340,7 +8616,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="72" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>285</v>
       </c>
@@ -8392,8 +8668,11 @@
       <c r="U72" t="s">
         <v>379</v>
       </c>
-    </row>
-    <row r="73" spans="1:24" hidden="1" x14ac:dyDescent="0.25">
+      <c r="V72" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="73" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>71</v>
       </c>
@@ -8437,7 +8716,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="74" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>127</v>
       </c>
@@ -8492,8 +8771,11 @@
       <c r="U74" t="s">
         <v>368</v>
       </c>
-    </row>
-    <row r="75" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="V74" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="75" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>193</v>
       </c>
@@ -8548,15 +8830,242 @@
       <c r="U75" t="s">
         <v>379</v>
       </c>
+      <c r="V75" t="s">
+        <v>331</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P75">
-    <filterColumn colId="11">
-      <filters>
-        <filter val="Pony Express Page 6"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:P75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B27"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="34.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B2" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>97</v>
+      </c>
+      <c r="B4" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>115</v>
+      </c>
+      <c r="B5" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>266</v>
+      </c>
+      <c r="B6" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>254</v>
+      </c>
+      <c r="B7" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>148</v>
+      </c>
+      <c r="B8" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>239</v>
+      </c>
+      <c r="B9" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>243</v>
+      </c>
+      <c r="B10" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>245</v>
+      </c>
+      <c r="B11" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>138</v>
+      </c>
+      <c r="B12" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>110</v>
+      </c>
+      <c r="B13" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>92</v>
+      </c>
+      <c r="B14" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>288</v>
+      </c>
+      <c r="B15" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>214</v>
+      </c>
+      <c r="B16" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>216</v>
+      </c>
+      <c r="B17" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>211</v>
+      </c>
+      <c r="B18" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>181</v>
+      </c>
+      <c r="B19" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>199</v>
+      </c>
+      <c r="B20" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>307</v>
+      </c>
+      <c r="B21" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>277</v>
+      </c>
+      <c r="B22" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>159</v>
+      </c>
+      <c r="B23" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>87</v>
+      </c>
+      <c r="B24" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>285</v>
+      </c>
+      <c r="B25" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>127</v>
+      </c>
+      <c r="B26" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>193</v>
+      </c>
+      <c r="B27" t="s">
+        <v>331</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>